<commit_message>
test-case-automation & qa & nfr-testing
</commit_message>
<xml_diff>
--- a/test-cases/test-cases.xlsx
+++ b/test-cases/test-cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\not99\Downloads\test-cases\test-cases\System Limits &amp; Vulnerability-test-cases - - Copy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\not99\Downloads\test-cases\test-cases\Automation, QA-test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632D00DE-745E-43F3-AB1D-DB66ECA5A9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E1FD57-6173-4510-9733-FA31EE82622F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D83949F6-E965-4507-AEDE-3C9312BAE01F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="258">
   <si>
     <t>Module</t>
   </si>
@@ -791,6 +791,78 @@
       </rPr>
       <t> ในช่องค้นหาและเอนเทอร์</t>
     </r>
+  </si>
+  <si>
+    <t>Manual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Auto.</t>
+  </si>
+  <si>
+    <t>Visual</t>
+  </si>
+  <si>
+    <t>Perf.</t>
+  </si>
+  <si>
+    <t>Auto.</t>
+  </si>
+  <si>
+    <t>Black Box &amp; Exploratory</t>
+  </si>
+  <si>
+    <t>Environment ปกติ</t>
+  </si>
+  <si>
+    <t>1. Manual Tester ทำการทดสอบโดยทดลอง input แปลกๆ และสุ่มกดเมนูต่างๆ</t>
+  </si>
+  <si>
+    <t>ตรวจพบ Edge Cases และ Bug ใหม่ๆ, สรุปผลทดสอบลงรายงาน</t>
+  </si>
+  <si>
+    <t>Playwright Tests (E2E)</t>
+  </si>
+  <si>
+    <t>เตรียม Playwright Script</t>
+  </si>
+  <si>
+    <t>1. Automation Engineer รันคำสั่งทดสอบ E2E Flow ของระบบทั้งหมด</t>
+  </si>
+  <si>
+    <t>Script รันผ่านสำเร็จ มี Test Report แจ้งผล Pass/Fail อัตโนมัติ</t>
+  </si>
+  <si>
+    <t>Visual &amp; Cross-browser</t>
+  </si>
+  <si>
+    <t>1. QA Analyst ตรวจสอบ UI บน Chrome, Edge, Safari และ Firefox</t>
+  </si>
+  <si>
+    <t>Components, สี, การจัดวางแสดงผลตรงตาม Design ไม่ผิดเพี้ยน</t>
+  </si>
+  <si>
+    <t>Load Testing (100 Users)</t>
+  </si>
+  <si>
+    <t>1. จำลองผู้ใช้งาน 100 คนค้นหาหนังสือและยืมคืนพร้อมกัน (อ้างอิง NFR 4.1)</t>
+  </si>
+  <si>
+    <t>ระบบทำงานได้ปกติ Response Time โดยเฉลี่ยไม่เกิน 2-3 วินาที</t>
+  </si>
+  <si>
+    <t>Backup / Failover Check</t>
+  </si>
+  <si>
+    <t>มีสิทธิ์เข้าถึงฝั่ง Server Docker</t>
+  </si>
+  <si>
+    <t>1. สั่ง Backup ฐานข้อมูล และจำลอง Database Crash (ปิด Container)</t>
+  </si>
+  <si>
+    <t>ข้อมูลกลับมาได้ครบถ้วนจากการกู้คืน ภายใน 4 ชม. ตาม NFR</t>
+  </si>
+  <si>
+    <t>ใช้เครื่องมือเช่น k6</t>
   </si>
 </sst>
 </file>
@@ -866,7 +938,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -883,6 +955,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1224,7 +1297,7 @@
     <col min="2" max="2" width="8.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="65.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="67.85546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="77.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="2"/>
@@ -2288,29 +2361,119 @@
         <v>77</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B47" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B48" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B49" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B50" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>76</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test-case-automation & qa & nfr-testing-2
</commit_message>
<xml_diff>
--- a/test-cases/test-cases.xlsx
+++ b/test-cases/test-cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\not99\Downloads\test-cases\test-cases\Automation, QA-test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E1FD57-6173-4510-9733-FA31EE82622F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8DD40D-1F5E-41AE-9301-F99B78D7096D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D83949F6-E965-4507-AEDE-3C9312BAE01F}"/>
   </bookViews>
@@ -2411,7 +2411,7 @@
       <c r="A49" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="2" t="s">
         <v>236</v>
       </c>
       <c r="C49" s="2" t="s">
@@ -2434,7 +2434,7 @@
       <c r="A50" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="5" t="s">
         <v>237</v>
       </c>
       <c r="C50" s="5" t="s">

</xml_diff>

<commit_message>
แก้ test-case-automation & qa & nfr-testing เป็น UI/UX
</commit_message>
<xml_diff>
--- a/test-cases/test-cases.xlsx
+++ b/test-cases/test-cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\not99\Downloads\test-cases\test-cases\Automation, QA-test-cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project wittawat\New folder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8DD40D-1F5E-41AE-9301-F99B78D7096D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4139EF25-A52C-4562-82CF-5AC4CAFC5941}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D83949F6-E965-4507-AEDE-3C9312BAE01F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="252">
   <si>
     <t>Module</t>
   </si>
@@ -793,76 +793,58 @@
     </r>
   </si>
   <si>
-    <t>Manual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">	Auto.</t>
-  </si>
-  <si>
-    <t>Visual</t>
-  </si>
-  <si>
-    <t>Perf.</t>
-  </si>
-  <si>
-    <t>Auto.</t>
-  </si>
-  <si>
-    <t>Black Box &amp; Exploratory</t>
-  </si>
-  <si>
-    <t>Environment ปกติ</t>
-  </si>
-  <si>
-    <t>1. Manual Tester ทำการทดสอบโดยทดลอง input แปลกๆ และสุ่มกดเมนูต่างๆ</t>
-  </si>
-  <si>
-    <t>ตรวจพบ Edge Cases และ Bug ใหม่ๆ, สรุปผลทดสอบลงรายงาน</t>
-  </si>
-  <si>
-    <t>Playwright Tests (E2E)</t>
-  </si>
-  <si>
-    <t>เตรียม Playwright Script</t>
-  </si>
-  <si>
-    <t>1. Automation Engineer รันคำสั่งทดสอบ E2E Flow ของระบบทั้งหมด</t>
-  </si>
-  <si>
-    <t>Script รันผ่านสำเร็จ มี Test Report แจ้งผล Pass/Fail อัตโนมัติ</t>
-  </si>
-  <si>
-    <t>Visual &amp; Cross-browser</t>
-  </si>
-  <si>
-    <t>1. QA Analyst ตรวจสอบ UI บน Chrome, Edge, Safari และ Firefox</t>
-  </si>
-  <si>
-    <t>Components, สี, การจัดวางแสดงผลตรงตาม Design ไม่ผิดเพี้ยน</t>
-  </si>
-  <si>
-    <t>Load Testing (100 Users)</t>
-  </si>
-  <si>
-    <t>1. จำลองผู้ใช้งาน 100 คนค้นหาหนังสือและยืมคืนพร้อมกัน (อ้างอิง NFR 4.1)</t>
-  </si>
-  <si>
-    <t>ระบบทำงานได้ปกติ Response Time โดยเฉลี่ยไม่เกิน 2-3 วินาที</t>
-  </si>
-  <si>
-    <t>Backup / Failover Check</t>
-  </si>
-  <si>
-    <t>มีสิทธิ์เข้าถึงฝั่ง Server Docker</t>
-  </si>
-  <si>
-    <t>1. สั่ง Backup ฐานข้อมูล และจำลอง Database Crash (ปิด Container)</t>
-  </si>
-  <si>
-    <t>ข้อมูลกลับมาได้ครบถ้วนจากการกู้คืน ภายใน 4 ชม. ตาม NFR</t>
-  </si>
-  <si>
-    <t>ใช้เครื่องมือเช่น k6</t>
+    <t>Toast Alert &amp; Feedback</t>
+  </si>
+  <si>
+    <t>1. ทำรายการไม่สำเร็จ เช่น คีย์รหัสหนังสือผิด</t>
+  </si>
+  <si>
+    <t>มุมจอแสดง Notification Popup แจ้ง Error สั้นๆ แล้วหายไป</t>
+  </si>
+  <si>
+    <t>Button Loading State</t>
+  </si>
+  <si>
+    <t>กดปุ่มทำงานหนัก / รอฐานข้อมูล</t>
+  </si>
+  <si>
+    <t>1. กดปุ่มบันทึก หรือส่งแบบฟอร์ม</t>
+  </si>
+  <si>
+    <t>ปุ่มจะแสดงสถานะ Loading Spinner และโดน Disable เพื่อป้องกันกดซ้ำ</t>
+  </si>
+  <si>
+    <t>Interactive Element Overlay</t>
+  </si>
+  <si>
+    <t>ชี้ Tooltip หรือคลิกเปิดปุ่ม Dropdown</t>
+  </si>
+  <si>
+    <t>1. ลองชี้เปิด Tooltip บนตารางส่วนต่างๆ</t>
+  </si>
+  <si>
+    <t>องค์ประกอบลอยตัวต้องโชว์เต็มบนสุด (Z-Index ถูกต้อง) ไม่มีอันอื่นมาซ้อนทับ</t>
+  </si>
+  <si>
+    <t>สีข้อความถูกปรับให้สว่างเพื่อให้มองเห็นได้ชัดเจนบนสีกราฟิกมืดทึบ</t>
+  </si>
+  <si>
+    <t>1. เดินดูเมนูต่างๆ ทั้ง Sidebar และกล่องค้นหา</t>
+  </si>
+  <si>
+    <t>ระบบปรับเป็นโหมดมืด (Dark Theme)</t>
+  </si>
+  <si>
+    <t>Dark Mode Display</t>
+  </si>
+  <si>
+    <t>Color Contrast Check</t>
+  </si>
+  <si>
+    <t>1. ตรวจสอบความเข้มของสีตัวอักษรและปุ่มต่างๆ เทียบกับสีพื้นหลัง</t>
+  </si>
+  <si>
+    <t>สบายตาผ่านเกณฑ์ Contrast Ratio ไม่กลืนไปกับพื้นหลังตาม Design System</t>
   </si>
 </sst>
 </file>
@@ -1296,7 +1278,7 @@
     <col min="1" max="1" width="6.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.140625" style="2" customWidth="1"/>
     <col min="5" max="5" width="67.85546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="77.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.7109375" style="2" bestFit="1" customWidth="1"/>
@@ -2366,22 +2348,22 @@
         <v>72</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>240</v>
+        <v>31</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2389,22 +2371,22 @@
         <v>73</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E48" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="C48" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>245</v>
-      </c>
       <c r="F48" s="3" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2412,42 +2394,42 @@
         <v>74</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>236</v>
+        <v>219</v>
       </c>
       <c r="C49" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="E49" s="6" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C50" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="C50" s="5" t="s">
-        <v>250</v>
-      </c>
       <c r="D50" s="5" t="s">
-        <v>257</v>
+        <v>238</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>77</v>
@@ -2458,19 +2440,19 @@
         <v>76</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>238</v>
+        <v>219</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>77</v>

</xml_diff>